<commit_message>
Fix win-rate tracker: stale SUM/COUNT range undercounts recent trades
K81/K82 (feeding the headline win-rate cell K80) are hardcoded to
J3:J72, so the 3 most recently resolved trades (rows 74, 75, 86) are
silently excluded - K80 shows 61.11% instead of the correct 59.65%.

There's already a second win-rate calc a few rows down (K84, via
K85/K86) that has the correct numbers (34/57) hand-entered as literal
values - so the two cells currently disagree with each other. Rather
than being two sources of truth that can drift apart again, K85/K86
now just reference the (corrected, self-extending) K81/K82, so both
cells always agree and stay correct as new trades are added.

Applied as a surgical patch to the formula/value cells only - every
other part of the file (styles, the external link to Biopharma.xlsx,
shared strings, etc.) is byte-for-byte unchanged.
</commit_message>
<xml_diff>
--- a/Recommendations.xlsx
+++ b/Recommendations.xlsx
@@ -2722,7 +2722,7 @@
       </c>
       <c r="K80" s="5">
         <f>+K81/K82</f>
-        <v>0.61111111111111116</v>
+        <v>0.59649122807017541</v>
       </c>
     </row>
     <row r="81" spans="2:12" x14ac:dyDescent="0.2">
@@ -2748,8 +2748,8 @@
         <v>86</v>
       </c>
       <c r="K81" s="4">
-        <f>SUM(J3:J72)</f>
-        <v>33</v>
+        <f>SUM(J3:J1000)</f>
+        <v>34</v>
       </c>
       <c r="L81" s="4">
         <f>+K82-K81</f>
@@ -2779,8 +2779,8 @@
         <v>86</v>
       </c>
       <c r="K82" s="4">
-        <f>COUNT(J3:J72)</f>
-        <v>54</v>
+        <f>COUNT(J3:J1000)</f>
+        <v>57</v>
       </c>
     </row>
     <row r="83" spans="2:12" x14ac:dyDescent="0.2">
@@ -2856,6 +2856,7 @@
         <v>83</v>
       </c>
       <c r="K85">
+        <f>K81</f>
         <v>34</v>
       </c>
       <c r="L85">
@@ -2886,6 +2887,7 @@
         <v>0</v>
       </c>
       <c r="K86">
+        <f>K82</f>
         <v>57</v>
       </c>
     </row>

</xml_diff>